<commit_message>
Adding module 3 assignment
</commit_message>
<xml_diff>
--- a/files/schedule_modules.xlsx
+++ b/files/schedule_modules.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jessicacooperstone/git/rdataviz/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC4A8C7-1E71-CF4D-84CB-D36E5B9D68E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65A3D25D-F80A-7944-8335-08D44F2380BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17480" yWindow="2380" windowWidth="28800" windowHeight="16360" activeTab="2" xr2:uid="{21EBE61F-A4F0-3D45-865A-9EB87E85AA6A}"/>
   </bookViews>
@@ -238,13 +238,13 @@
     <t>Tuesday, December 8, 2026</t>
   </si>
   <si>
-    <t>Tuesday, November 10, 2026</t>
-  </si>
-  <si>
     <t>Sunday, December 13, 2026</t>
   </si>
   <si>
     <t>due_date_paste</t>
+  </si>
+  <si>
+    <t>Tuesday, November 17, 2026</t>
   </si>
 </sst>
 </file>
@@ -986,10 +986,10 @@
         <v>46329</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="D12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -1000,10 +1000,10 @@
         <v>46336</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>53</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H13" s="2"/>
     </row>
@@ -1093,7 +1093,7 @@
         <v>25</v>
       </c>
       <c r="C1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -1171,11 +1171,11 @@
         <v>31</v>
       </c>
       <c r="B8" s="5">
-        <f>Schedule_date_2026!B13</f>
-        <v>46336</v>
+        <f>Schedule_date_2026!B14</f>
+        <v>46343</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -1187,7 +1187,7 @@
         <v>46369</v>
       </c>
       <c r="C9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>